<commit_message>
Adiciona produtos de exemplo à planilha
</commit_message>
<xml_diff>
--- a/BM_MOTOS_Gestao_Estoque_Caixa_Template.xlsx
+++ b/BM_MOTOS_Gestao_Estoque_Caixa_Template.xlsx
@@ -15,14 +15,18 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mecanicos" sheetId="6" state="hidden" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Caixa" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Produtos'!$A$1:$G$21</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="R$ #,##0.00"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -41,7 +45,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -52,6 +56,11 @@
       <patternFill patternType="solid">
         <fgColor rgb="002F5496"/>
         <bgColor rgb="002F5496"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
   </fills>
@@ -73,12 +82,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -468,56 +482,637 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>ID_Produto</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Categoria</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Preco_Custo</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Preco_Venda</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>Quantidade</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>Unidade</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Óleo para motor 10W40 1L</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Óleos e Lubrificantes</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Litro</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Óleo para motor 20W50 1L</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Óleos e Lubrificantes</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Litro</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Fluido de freio DOT 4 500ml</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Freios</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="E4" s="5" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Un</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Filtro de óleo universal</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Filtros</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>24.9</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Un</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Filtro de ar CG 160</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Filtros</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Un</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Pastilha de freio dianteira</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Freios</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Jogo</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Lona de freio traseira</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Freios</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>54.9</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Jogo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Vela de ignição NGK</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Ignição</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Un</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Cabo de embreagem universal</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Cabos</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Un</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Cabo de acelerador universal</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Cabos</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Un</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Kit relação CG 160</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Transmissão</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>118</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>189.9</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Jogo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Corrente de transmissão 428H</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Transmissão</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>65</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>109.9</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Un</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Pneu dianteiro 90/90-18</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Pneus</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>148</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>239.9</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Un</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Pneu traseiro 100/80-18</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Pneus</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>205</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>329.9</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Un</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Câmara de ar aro 18</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Pneus</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Un</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Lâmpada de farol H4 35/35W</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Elétrica</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="F17" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Un</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Bateria 12V 6Ah</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Elétrica</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>180</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>279.9</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Un</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Kit de lâmpadas e fusíveis</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Elétrica</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Jogo</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Rolamento de roda dianteira</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Suspensão</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>24</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>44.9</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Un</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Graxa branca spray 300ml</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Óleos e Lubrificantes</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>34.9</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Un</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:G21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Adiciona mecanicos de exemplo com senhas protegidas
</commit_message>
<xml_diff>
--- a/BM_MOTOS_Gestao_Estoque_Caixa_Template.xlsx
+++ b/BM_MOTOS_Gestao_Estoque_Caixa_Template.xlsx
@@ -17,6 +17,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Produtos'!$A$1:$G$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Mecanicos'!$A$1:$D$3</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1309,38 +1310,79 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="95" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>ID_Mecanico</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>Nome</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Telefone</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Senha</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Mecânico Exemplo 1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Não informado</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>pbkdf2_sha256$200000$17dd554025da04ad0caccaea6457dd87$6be575f8ec57db943fad1848ea62b97b64e231af91ce9bfced04948a3e8ffe77</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Mecânico Exemplo 2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Não informado</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>pbkdf2_sha256$200000$3c0e2dc5a38985728c45a345c997af50$c73b1cb91fb8492ddb12d6226223ca2f6431e698988ab6df851268799c9d5285</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:D3"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>